<commit_message>
Add 32 Potenza questionnaires and refresh reports
</commit_message>
<xml_diff>
--- a/data/LIC2026/questionari.xlsx
+++ b/data/LIC2026/questionari.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dati codificati" sheetId="1" r:id="R7b33a635471d48f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risposte originali" sheetId="2" r:id="R4fb013f3f3f5414c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dati codificati" sheetId="1" r:id="R81d35f6573c84259"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risposte originali" sheetId="2" r:id="Rc6609a7570354e7a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -83,18 +83,25 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="2">
+  <x:dxfs count="3">
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F1DC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF0C2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFFF0C2"/>
+          <x:bgColor rgb="FFE8F1DC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -103,7 +110,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DatiHEPscape" displayName="DatiHEPscape" ref="A6:O87" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DatiHEPscape" displayName="DatiHEPscape" ref="A6:O119" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="15">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Q1"/>
@@ -126,7 +133,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="OriginaliHEPscape" displayName="OriginaliHEPscape" ref="A1:S82" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="OriginaliHEPscape" displayName="OriginaliHEPscape" ref="A1:S114" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="19">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Q1"/>
@@ -366,7 +373,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>HEPscape! | Lucania is comics | 81 questionari</x:v>
+        <x:v>HEPscape! | Lucania is comics | 113 questionari</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
@@ -4400,6 +4407,1510 @@
         <x:v>Lucania is comics</x:v>
       </x:c>
     </x:row>
+    <x:row r="88" ht="34" customHeight="1">
+      <x:c r="A88" s="3" t="str">
+        <x:v>LIC2026-IMG2537</x:v>
+      </x:c>
+      <x:c r="B88" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C88" s="3" t="n">
+        <x:v>999</x:v>
+      </x:c>
+      <x:c r="D88" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E88" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F88" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G88" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H88" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I88" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J88" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K88" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L88" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M88" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N88" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O88" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="34" customHeight="1">
+      <x:c r="A89" s="3" t="str">
+        <x:v>LIC2026-IMG2538</x:v>
+      </x:c>
+      <x:c r="B89" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C89" s="3" t="str">
+        <x:v>DIVERTENTE - APPASSIONANTE</x:v>
+      </x:c>
+      <x:c r="D89" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E89" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F89" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G89" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H89" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I89" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J89" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K89" s="3" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="L89" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M89" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N89" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O89" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="34" customHeight="1">
+      <x:c r="A90" s="3" t="str">
+        <x:v>LIC2026-IMG2539</x:v>
+      </x:c>
+      <x:c r="B90" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C90" s="3" t="str">
+        <x:v>INTERESSANTE</x:v>
+      </x:c>
+      <x:c r="D90" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E90" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F90" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G90" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H90" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I90" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J90" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K90" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L90" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M90" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N90" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O90" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="34" customHeight="1">
+      <x:c r="A91" s="3" t="str">
+        <x:v>LIC2026-IMG2540</x:v>
+      </x:c>
+      <x:c r="B91" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C91" s="3" t="str">
+        <x:v>INTERESSANTE</x:v>
+      </x:c>
+      <x:c r="D91" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E91" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F91" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G91" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H91" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I91" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J91" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K91" s="3" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="L91" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M91" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N91" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O91" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="34" customHeight="1">
+      <x:c r="A92" s="3" t="str">
+        <x:v>LIC2026-IMG2541</x:v>
+      </x:c>
+      <x:c r="B92" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C92" s="3" t="str">
+        <x:v>COINVOLGENTE E INTERESSANTE</x:v>
+      </x:c>
+      <x:c r="D92" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E92" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F92" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G92" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H92" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I92" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J92" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K92" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L92" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M92" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N92" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O92" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="34" customHeight="1">
+      <x:c r="A93" s="3" t="str">
+        <x:v>LIC2026-IMG2542</x:v>
+      </x:c>
+      <x:c r="B93" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C93" s="3" t="str">
+        <x:v>CURIOSA SCIENTIFICA PROFESSIONALE</x:v>
+      </x:c>
+      <x:c r="D93" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E93" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F93" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G93" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H93" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I93" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J93" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K93" s="3" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="L93" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M93" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N93" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O93" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="34" customHeight="1">
+      <x:c r="A94" s="3" t="str">
+        <x:v>LIC2026-IMG2543</x:v>
+      </x:c>
+      <x:c r="B94" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C94" s="3" t="str">
+        <x:v>CARINA, INTERATTIVA, SIMPATICA</x:v>
+      </x:c>
+      <x:c r="D94" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E94" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F94" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G94" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H94" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I94" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J94" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K94" s="3" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L94" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M94" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N94" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O94" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="34" customHeight="1">
+      <x:c r="A95" s="3" t="str">
+        <x:v>LIC2026-IMG2544</x:v>
+      </x:c>
+      <x:c r="B95" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C95" s="3" t="str">
+        <x:v>INTERESSANTE, CURIOSO, SORPRENDENTE</x:v>
+      </x:c>
+      <x:c r="D95" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E95" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F95" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G95" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H95" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I95" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J95" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K95" s="3" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L95" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M95" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N95" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O95" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="34" customHeight="1">
+      <x:c r="A96" s="3" t="str">
+        <x:v>LIC2026-IMG2545</x:v>
+      </x:c>
+      <x:c r="B96" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C96" s="3" t="str">
+        <x:v>STIMOLANTE ISTRUTTIVO DIVERTENTE</x:v>
+      </x:c>
+      <x:c r="D96" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E96" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F96" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G96" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H96" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I96" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J96" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K96" s="3" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L96" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M96" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N96" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O96" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="34" customHeight="1">
+      <x:c r="A97" s="3" t="str">
+        <x:v>LIC2026-IMG2546</x:v>
+      </x:c>
+      <x:c r="B97" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C97" s="3" t="str">
+        <x:v>DIVERTENTE, SIMPATICA, ISTRUTTIVA</x:v>
+      </x:c>
+      <x:c r="D97" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E97" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F97" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G97" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H97" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I97" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J97" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K97" s="3" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L97" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M97" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N97" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O97" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="34" customHeight="1">
+      <x:c r="A98" s="3" t="str">
+        <x:v>LIC2026-IMG2547</x:v>
+      </x:c>
+      <x:c r="B98" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C98" s="3" t="str">
+        <x:v>MOLTO INTERESSANTE</x:v>
+      </x:c>
+      <x:c r="D98" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E98" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F98" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G98" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H98" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I98" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J98" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K98" s="3" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L98" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M98" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N98" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O98" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="34" customHeight="1">
+      <x:c r="A99" s="3" t="str">
+        <x:v>LIC2026-IMG2548</x:v>
+      </x:c>
+      <x:c r="B99" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C99" s="3" t="str">
+        <x:v>COINVOLGENTE, DIVERTENTE,</x:v>
+      </x:c>
+      <x:c r="D99" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E99" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F99" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G99" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H99" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I99" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J99" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K99" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L99" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M99" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N99" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O99" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="34" customHeight="1">
+      <x:c r="A100" s="3" t="str">
+        <x:v>LIC2026-IMG2549</x:v>
+      </x:c>
+      <x:c r="B100" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C100" s="3" t="str">
+        <x:v>BELLO, INTERESSANTE</x:v>
+      </x:c>
+      <x:c r="D100" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E100" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F100" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G100" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H100" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I100" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J100" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K100" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L100" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M100" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N100" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O100" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="34" customHeight="1">
+      <x:c r="A101" s="3" t="str">
+        <x:v>LIC2026-IMG2550</x:v>
+      </x:c>
+      <x:c r="B101" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C101" s="3" t="n">
+        <x:v>999</x:v>
+      </x:c>
+      <x:c r="D101" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E101" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F101" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G101" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H101" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I101" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J101" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K101" s="3" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="L101" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M101" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N101" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O101" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="34" customHeight="1">
+      <x:c r="A102" s="3" t="str">
+        <x:v>LIC2026-IMG2553</x:v>
+      </x:c>
+      <x:c r="B102" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C102" s="3" t="str">
+        <x:v>BELLA, INTERESSANTE, COINVOLGENTE</x:v>
+      </x:c>
+      <x:c r="D102" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E102" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F102" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G102" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H102" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I102" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J102" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K102" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L102" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M102" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N102" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O102" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="34" customHeight="1">
+      <x:c r="A103" s="3" t="str">
+        <x:v>LIC2026-IMG2554</x:v>
+      </x:c>
+      <x:c r="B103" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C103" s="3" t="str">
+        <x:v>RAGIONAMENTO, ATTENZIONE, SCOPERTA</x:v>
+      </x:c>
+      <x:c r="D103" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E103" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F103" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G103" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H103" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I103" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J103" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K103" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L103" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M103" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N103" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O103" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="34" customHeight="1">
+      <x:c r="A104" s="3" t="str">
+        <x:v>LIC2026-IMG2555</x:v>
+      </x:c>
+      <x:c r="B104" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C104" s="3" t="str">
+        <x:v>DIVULGATIVA</x:v>
+      </x:c>
+      <x:c r="D104" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E104" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F104" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G104" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H104" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I104" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J104" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K104" s="3" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L104" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M104" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N104" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O104" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="34" customHeight="1">
+      <x:c r="A105" s="3" t="str">
+        <x:v>LIC2026-IMG2556</x:v>
+      </x:c>
+      <x:c r="B105" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C105" s="3" t="str">
+        <x:v>INTERATTIVA</x:v>
+      </x:c>
+      <x:c r="D105" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E105" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F105" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G105" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H105" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I105" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J105" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K105" s="3" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L105" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M105" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N105" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O105" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="34" customHeight="1">
+      <x:c r="A106" s="3" t="str">
+        <x:v>LIC2026-IMG2557</x:v>
+      </x:c>
+      <x:c r="B106" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C106" s="3" t="str">
+        <x:v>ORIGINALE, COINVOLGENTE</x:v>
+      </x:c>
+      <x:c r="D106" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E106" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F106" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G106" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H106" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I106" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J106" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K106" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L106" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M106" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N106" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O106" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="34" customHeight="1">
+      <x:c r="A107" s="3" t="str">
+        <x:v>LIC2026-IMG2558</x:v>
+      </x:c>
+      <x:c r="B107" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C107" s="3" t="str">
+        <x:v>INTERESSANTE</x:v>
+      </x:c>
+      <x:c r="D107" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E107" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F107" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G107" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H107" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I107" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J107" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K107" s="3" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L107" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M107" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N107" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O107" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="34" customHeight="1">
+      <x:c r="A108" s="3" t="str">
+        <x:v>LIC2026-IMG2559</x:v>
+      </x:c>
+      <x:c r="B108" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C108" s="3" t="n">
+        <x:v>999</x:v>
+      </x:c>
+      <x:c r="D108" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E108" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F108" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G108" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H108" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I108" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J108" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K108" s="3" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="L108" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M108" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N108" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O108" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="34" customHeight="1">
+      <x:c r="A109" s="3" t="str">
+        <x:v>LIC2026-IMG2560</x:v>
+      </x:c>
+      <x:c r="B109" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C109" s="3" t="str">
+        <x:v>DIVERTENTE, EDUCATIVA</x:v>
+      </x:c>
+      <x:c r="D109" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E109" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F109" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G109" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H109" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I109" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J109" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K109" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L109" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M109" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N109" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O109" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="34" customHeight="1">
+      <x:c r="A110" s="3" t="str">
+        <x:v>LIC2026-IMG2561</x:v>
+      </x:c>
+      <x:c r="B110" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C110" s="3" t="str">
+        <x:v>DIVERTENTE, STIMOLANTE</x:v>
+      </x:c>
+      <x:c r="D110" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E110" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F110" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G110" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H110" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I110" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J110" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K110" s="3" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="L110" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M110" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N110" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O110" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="34" customHeight="1">
+      <x:c r="A111" s="3" t="str">
+        <x:v>LIC2026-IMG2562</x:v>
+      </x:c>
+      <x:c r="B111" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C111" s="3" t="n">
+        <x:v>999</x:v>
+      </x:c>
+      <x:c r="D111" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E111" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F111" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G111" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H111" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I111" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J111" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K111" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L111" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M111" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N111" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O111" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="34" customHeight="1">
+      <x:c r="A112" s="3" t="str">
+        <x:v>LIC2026-IMG2563</x:v>
+      </x:c>
+      <x:c r="B112" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C112" s="3" t="n">
+        <x:v>999</x:v>
+      </x:c>
+      <x:c r="D112" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E112" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F112" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G112" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H112" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I112" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J112" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K112" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L112" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M112" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N112" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O112" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="34" customHeight="1">
+      <x:c r="A113" s="3" t="str">
+        <x:v>LIC2026-IMG2564</x:v>
+      </x:c>
+      <x:c r="B113" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C113" s="3" t="str">
+        <x:v>DIVERTENTE, COLLABORATIVA</x:v>
+      </x:c>
+      <x:c r="D113" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E113" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F113" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G113" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H113" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I113" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J113" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K113" s="3" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L113" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M113" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N113" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O113" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="34" customHeight="1">
+      <x:c r="A114" s="3" t="str">
+        <x:v>LIC2026-IMG2565</x:v>
+      </x:c>
+      <x:c r="B114" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C114" s="3" t="n">
+        <x:v>999</x:v>
+      </x:c>
+      <x:c r="D114" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E114" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F114" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G114" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H114" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I114" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J114" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K114" s="3" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L114" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M114" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N114" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O114" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="34" customHeight="1">
+      <x:c r="A115" s="3" t="str">
+        <x:v>LIC2026-IMG2566</x:v>
+      </x:c>
+      <x:c r="B115" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C115" s="3" t="str">
+        <x:v>DIVERTENTE EDUCATIVA</x:v>
+      </x:c>
+      <x:c r="D115" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E115" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F115" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G115" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H115" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I115" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J115" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K115" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L115" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M115" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N115" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O115" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="34" customHeight="1">
+      <x:c r="A116" s="3" t="str">
+        <x:v>LIC2026-IMG2568</x:v>
+      </x:c>
+      <x:c r="B116" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C116" s="3" t="str">
+        <x:v>FIGO ASSAI</x:v>
+      </x:c>
+      <x:c r="D116" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E116" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F116" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G116" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H116" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I116" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J116" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K116" s="3" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L116" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M116" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N116" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O116" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="34" customHeight="1">
+      <x:c r="A117" s="3" t="str">
+        <x:v>LIC2026-IMG2570</x:v>
+      </x:c>
+      <x:c r="B117" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C117" s="3" t="str">
+        <x:v>INGEGNERISTICA SUPER QUARK</x:v>
+      </x:c>
+      <x:c r="D117" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E117" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F117" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G117" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H117" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I117" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J117" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K117" s="3" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L117" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M117" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N117" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O117" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="34" customHeight="1">
+      <x:c r="A118" s="3" t="str">
+        <x:v>LIC2026-IMG2571</x:v>
+      </x:c>
+      <x:c r="B118" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C118" s="3" t="str">
+        <x:v>BELLA CURIOSA DIVERTENTE</x:v>
+      </x:c>
+      <x:c r="D118" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E118" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F118" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G118" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H118" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I118" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J118" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K118" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L118" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M118" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N118" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O118" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="34" customHeight="1">
+      <x:c r="A119" s="3" t="str">
+        <x:v>LIC2026-IMG2572</x:v>
+      </x:c>
+      <x:c r="B119" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C119" s="3" t="n">
+        <x:v>999</x:v>
+      </x:c>
+      <x:c r="D119" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E119" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F119" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G119" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H119" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I119" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J119" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K119" s="3" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="L119" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M119" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="N119" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="O119" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:O1"/>
@@ -4410,7 +5921,12 @@
     </x:cfRule>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="DA VERIFICARE"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="10">
+  <x:conditionalFormatting sqref="B88:L119">
+    <x:cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+      <x:formula>999</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:dataValidations count="20">
     <x:dataValidation type="list" sqref="B7:B87">
       <x:formula1>"0,1,2,999"</x:formula1>
     </x:dataValidation>
@@ -4441,10 +5957,40 @@
     <x:dataValidation type="list" sqref="L7:L87">
       <x:formula1>"0,1,999"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="B88:B119">
+      <x:formula1>"0,1,2,999"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D88:D119">
+      <x:formula1>"0,1,2,999"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="E88:E119">
+      <x:formula1>"0,1,2,999"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="F88:F119">
+      <x:formula1>"0,1,2,999"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="G88:G119">
+      <x:formula1>"0,1,2,999"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="H88:H119">
+      <x:formula1>"0,1,2,999"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I88:I119">
+      <x:formula1>"0,1,999"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="J88:J119">
+      <x:formula1>"0,1,2,3,999"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="K88:K119">
+      <x:formula1>"0,1,2,3,4,5,6,7,999"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="L88:L119">
+      <x:formula1>"0,1,999"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R527752675c2d47e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R085b50e6d4f94510"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9294,10 +10840,1892 @@
         <x:v>Lucania is comics</x:v>
       </x:c>
     </x:row>
+    <x:row r="83" ht="40" customHeight="1">
+      <x:c r="A83" s="3" t="str">
+        <x:v>LIC2026-IMG2537</x:v>
+      </x:c>
+      <x:c r="B83" s="3" t="str">
+        <x:v>Mi è piaciuta tantissimo</x:v>
+      </x:c>
+      <x:c r="C83" s="3" t="str"/>
+      <x:c r="D83" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="E83" s="3" t="str">
+        <x:v>Più curioso/a</x:v>
+      </x:c>
+      <x:c r="F83" s="3" t="str">
+        <x:v>Più interessato/a</x:v>
+      </x:c>
+      <x:c r="G83" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="H83" s="3" t="str">
+        <x:v>A volte</x:v>
+      </x:c>
+      <x:c r="I83" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J83" s="3" t="str">
+        <x:v>Maschile</x:v>
+      </x:c>
+      <x:c r="K83" s="3" t="str">
+        <x:v>15–18</x:v>
+      </x:c>
+      <x:c r="L83" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="M83" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 113
+Q2: Risposta non compilata nella fotografia.</x:v>
+      </x:c>
+      <x:c r="N83" s="3" t="str">
+        <x:v>IMG_2537.JPG</x:v>
+      </x:c>
+      <x:c r="O83" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P83" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q83" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R83" s="3" t="str">
+        <x:v>27d77079d4e002f17b48644c5324af01f61839742910170881f393738cea3e81</x:v>
+      </x:c>
+      <x:c r="S83" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="40" customHeight="1">
+      <x:c r="A84" s="3" t="str">
+        <x:v>LIC2026-IMG2538</x:v>
+      </x:c>
+      <x:c r="B84" s="3" t="str">
+        <x:v>Mi è piaciuta tantissimo</x:v>
+      </x:c>
+      <x:c r="C84" s="3" t="str">
+        <x:v>DIVERTENTE - APPASSIONANTE</x:v>
+      </x:c>
+      <x:c r="D84" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="E84" s="3" t="str">
+        <x:v>Curioso/a come prima</x:v>
+      </x:c>
+      <x:c r="F84" s="3" t="str">
+        <x:v>Interessato/a come prima</x:v>
+      </x:c>
+      <x:c r="G84" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="H84" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I84" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="J84" s="3" t="str">
+        <x:v>Maschile</x:v>
+      </x:c>
+      <x:c r="K84" s="3" t="str">
+        <x:v>41–60</x:v>
+      </x:c>
+      <x:c r="L84" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="M84" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 112</x:v>
+      </x:c>
+      <x:c r="N84" s="3" t="str">
+        <x:v>IMG_2538.JPG</x:v>
+      </x:c>
+      <x:c r="O84" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P84" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q84" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R84" s="3" t="str">
+        <x:v>5d4e3fd57b1964a99468da61d1eca8b27cef11539eaa756a0c3221ae80baa41a</x:v>
+      </x:c>
+      <x:c r="S84" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="40" customHeight="1">
+      <x:c r="A85" s="3" t="str">
+        <x:v>LIC2026-IMG2539</x:v>
+      </x:c>
+      <x:c r="B85" s="3" t="str">
+        <x:v>Mi è piaciuta tantissimo</x:v>
+      </x:c>
+      <x:c r="C85" s="3" t="str">
+        <x:v>Interessante</x:v>
+      </x:c>
+      <x:c r="D85" s="3" t="str">
+        <x:v>Sì, un po’</x:v>
+      </x:c>
+      <x:c r="E85" s="3" t="str">
+        <x:v>Curioso/a come prima</x:v>
+      </x:c>
+      <x:c r="F85" s="3" t="str">
+        <x:v>Interessato/a come prima</x:v>
+      </x:c>
+      <x:c r="G85" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="H85" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I85" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="J85" s="3" t="str">
+        <x:v>Maschile</x:v>
+      </x:c>
+      <x:c r="K85" s="3" t="str">
+        <x:v>15–18</x:v>
+      </x:c>
+      <x:c r="L85" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="M85" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 111</x:v>
+      </x:c>
+      <x:c r="N85" s="3" t="str">
+        <x:v>IMG_2539.JPG</x:v>
+      </x:c>
+      <x:c r="O85" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P85" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q85" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R85" s="3" t="str">
+        <x:v>a550714f2602bfd1b13fd98c81d98199ab82815ddada868299ac90d57f9a5e43</x:v>
+      </x:c>
+      <x:c r="S85" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="40" customHeight="1">
+      <x:c r="A86" s="3" t="str">
+        <x:v>LIC2026-IMG2540</x:v>
+      </x:c>
+      <x:c r="B86" s="3" t="str">
+        <x:v>Mi è piaciuta</x:v>
+      </x:c>
+      <x:c r="C86" s="3" t="str">
+        <x:v>INTERESSANTE</x:v>
+      </x:c>
+      <x:c r="D86" s="3" t="str">
+        <x:v>Sì, un po’</x:v>
+      </x:c>
+      <x:c r="E86" s="3" t="str">
+        <x:v>Più curioso/a</x:v>
+      </x:c>
+      <x:c r="F86" s="3" t="str">
+        <x:v>Più interessato/a</x:v>
+      </x:c>
+      <x:c r="G86" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="H86" s="3" t="str">
+        <x:v>A volte</x:v>
+      </x:c>
+      <x:c r="I86" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J86" s="3" t="str">
+        <x:v>Maschile</x:v>
+      </x:c>
+      <x:c r="K86" s="3" t="str">
+        <x:v>41–60</x:v>
+      </x:c>
+      <x:c r="L86" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="M86" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 110</x:v>
+      </x:c>
+      <x:c r="N86" s="3" t="str">
+        <x:v>IMG_2540.JPG</x:v>
+      </x:c>
+      <x:c r="O86" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P86" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q86" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R86" s="3" t="str">
+        <x:v>c164d871be15983edc5452997c11a1d7b93a6d7739c749df99465fccd416c7e4</x:v>
+      </x:c>
+      <x:c r="S86" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="40" customHeight="1">
+      <x:c r="A87" s="3" t="str">
+        <x:v>LIC2026-IMG2541</x:v>
+      </x:c>
+      <x:c r="B87" s="3" t="str">
+        <x:v>Mi è piaciuta tantissimo</x:v>
+      </x:c>
+      <x:c r="C87" s="3" t="str">
+        <x:v>COINVOLGENTE E INTERESSANTE</x:v>
+      </x:c>
+      <x:c r="D87" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="E87" s="3" t="str">
+        <x:v>Curioso/a come prima</x:v>
+      </x:c>
+      <x:c r="F87" s="3" t="str">
+        <x:v>Più interessato/a</x:v>
+      </x:c>
+      <x:c r="G87" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="H87" s="3" t="str">
+        <x:v>A volte</x:v>
+      </x:c>
+      <x:c r="I87" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="J87" s="3" t="str">
+        <x:v>Femminile</x:v>
+      </x:c>
+      <x:c r="K87" s="3" t="str">
+        <x:v>11–14</x:v>
+      </x:c>
+      <x:c r="L87" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="M87" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 109</x:v>
+      </x:c>
+      <x:c r="N87" s="3" t="str">
+        <x:v>IMG_2541.JPG</x:v>
+      </x:c>
+      <x:c r="O87" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P87" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q87" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R87" s="3" t="str">
+        <x:v>4d34e94a3a687abf9f02eb2183e201f1b06a68d3680ec5273704c48009a207c9</x:v>
+      </x:c>
+      <x:c r="S87" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="40" customHeight="1">
+      <x:c r="A88" s="3" t="str">
+        <x:v>LIC2026-IMG2542</x:v>
+      </x:c>
+      <x:c r="B88" s="3" t="str">
+        <x:v>Mi è piaciuta tantissimo</x:v>
+      </x:c>
+      <x:c r="C88" s="3" t="str">
+        <x:v>CURIOSA SCIENTIFICA PROFESSIONALE</x:v>
+      </x:c>
+      <x:c r="D88" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="E88" s="3" t="str">
+        <x:v>Più curioso/a</x:v>
+      </x:c>
+      <x:c r="F88" s="3" t="str">
+        <x:v>Più interessato/a</x:v>
+      </x:c>
+      <x:c r="G88" s="3" t="str">
+        <x:v>In parte</x:v>
+      </x:c>
+      <x:c r="H88" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I88" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="J88" s="3" t="str">
+        <x:v>Femminile</x:v>
+      </x:c>
+      <x:c r="K88" s="3" t="str">
+        <x:v>41–60</x:v>
+      </x:c>
+      <x:c r="L88" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="M88" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 108</x:v>
+      </x:c>
+      <x:c r="N88" s="3" t="str">
+        <x:v>IMG_2542.JPG</x:v>
+      </x:c>
+      <x:c r="O88" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P88" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q88" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R88" s="3" t="str">
+        <x:v>d9d025c43f0bab24a095b9a1990e05bc8fb2797412dfcf05d05dbc6e73bc6936</x:v>
+      </x:c>
+      <x:c r="S88" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="40" customHeight="1">
+      <x:c r="A89" s="3" t="str">
+        <x:v>LIC2026-IMG2543</x:v>
+      </x:c>
+      <x:c r="B89" s="3" t="str">
+        <x:v>Mi è piaciuta</x:v>
+      </x:c>
+      <x:c r="C89" s="3" t="str">
+        <x:v>CARINA, INTERATTIVA, SIMPATICA</x:v>
+      </x:c>
+      <x:c r="D89" s="3" t="str">
+        <x:v>Sì, un po’</x:v>
+      </x:c>
+      <x:c r="E89" s="3" t="str">
+        <x:v>Più curioso/a</x:v>
+      </x:c>
+      <x:c r="F89" s="3" t="str">
+        <x:v>Più interessato/a</x:v>
+      </x:c>
+      <x:c r="G89" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="H89" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I89" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J89" s="3" t="str">
+        <x:v>Femminile</x:v>
+      </x:c>
+      <x:c r="K89" s="3" t="str">
+        <x:v>19–25</x:v>
+      </x:c>
+      <x:c r="L89" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="M89" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 107</x:v>
+      </x:c>
+      <x:c r="N89" s="3" t="str">
+        <x:v>IMG_2543.JPG</x:v>
+      </x:c>
+      <x:c r="O89" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P89" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q89" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R89" s="3" t="str">
+        <x:v>63ee7e81b39aa6ee78a2b6b4bf3caeb4ec77fd1431ffe1c05c33d41b26b21924</x:v>
+      </x:c>
+      <x:c r="S89" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="40" customHeight="1">
+      <x:c r="A90" s="3" t="str">
+        <x:v>LIC2026-IMG2544</x:v>
+      </x:c>
+      <x:c r="B90" s="3" t="str">
+        <x:v>Mi è piaciuta tantissimo</x:v>
+      </x:c>
+      <x:c r="C90" s="3" t="str">
+        <x:v>INTERESSANTE, CURIOSO, SORPRENDENTE</x:v>
+      </x:c>
+      <x:c r="D90" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="E90" s="3" t="str">
+        <x:v>Più curioso/a</x:v>
+      </x:c>
+      <x:c r="F90" s="3" t="str">
+        <x:v>Più interessato/a</x:v>
+      </x:c>
+      <x:c r="G90" s="3" t="str">
+        <x:v>In parte</x:v>
+      </x:c>
+      <x:c r="H90" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I90" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J90" s="3" t="str">
+        <x:v>Femminile</x:v>
+      </x:c>
+      <x:c r="K90" s="3" t="str">
+        <x:v>19–25</x:v>
+      </x:c>
+      <x:c r="L90" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="M90" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 106</x:v>
+      </x:c>
+      <x:c r="N90" s="3" t="str">
+        <x:v>IMG_2544.JPG</x:v>
+      </x:c>
+      <x:c r="O90" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P90" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q90" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R90" s="3" t="str">
+        <x:v>cd5af2f60f719207d1f70d90ef192319ef04dd2d8abbb1f28590fcaee27c14ee</x:v>
+      </x:c>
+      <x:c r="S90" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="40" customHeight="1">
+      <x:c r="A91" s="3" t="str">
+        <x:v>LIC2026-IMG2545</x:v>
+      </x:c>
+      <x:c r="B91" s="3" t="str">
+        <x:v>Mi è piaciuta tantissimo</x:v>
+      </x:c>
+      <x:c r="C91" s="3" t="str">
+        <x:v>STIMOLANTE ISTRUTTIVO DIVERTENTE</x:v>
+      </x:c>
+      <x:c r="D91" s="3" t="str">
+        <x:v>Sì, un po’</x:v>
+      </x:c>
+      <x:c r="E91" s="3" t="str">
+        <x:v>Più curioso/a</x:v>
+      </x:c>
+      <x:c r="F91" s="3" t="str">
+        <x:v>Più interessato/a</x:v>
+      </x:c>
+      <x:c r="G91" s="3" t="str">
+        <x:v>In parte</x:v>
+      </x:c>
+      <x:c r="H91" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I91" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J91" s="3" t="str">
+        <x:v>Femminile</x:v>
+      </x:c>
+      <x:c r="K91" s="3" t="str">
+        <x:v>26–40</x:v>
+      </x:c>
+      <x:c r="L91" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="M91" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 105</x:v>
+      </x:c>
+      <x:c r="N91" s="3" t="str">
+        <x:v>IMG_2545.JPG</x:v>
+      </x:c>
+      <x:c r="O91" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P91" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q91" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R91" s="3" t="str">
+        <x:v>23358be92ef19092640404e999aaebb6404d0e4e2f11a9cf5b4453a7ee32019d</x:v>
+      </x:c>
+      <x:c r="S91" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="40" customHeight="1">
+      <x:c r="A92" s="3" t="str">
+        <x:v>LIC2026-IMG2546</x:v>
+      </x:c>
+      <x:c r="B92" s="3" t="str">
+        <x:v>Mi è piaciuta</x:v>
+      </x:c>
+      <x:c r="C92" s="3" t="str">
+        <x:v>DIVERTENTE, SIMPATICA, ISTRUTTIVA</x:v>
+      </x:c>
+      <x:c r="D92" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="E92" s="3" t="str">
+        <x:v>Curioso/a come prima</x:v>
+      </x:c>
+      <x:c r="F92" s="3" t="str">
+        <x:v>Più interessato/a</x:v>
+      </x:c>
+      <x:c r="G92" s="3" t="str">
+        <x:v>In parte</x:v>
+      </x:c>
+      <x:c r="H92" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I92" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J92" s="3" t="str">
+        <x:v>Femminile</x:v>
+      </x:c>
+      <x:c r="K92" s="3" t="str">
+        <x:v>26–40</x:v>
+      </x:c>
+      <x:c r="L92" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="M92" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 104</x:v>
+      </x:c>
+      <x:c r="N92" s="3" t="str">
+        <x:v>IMG_2546.JPG</x:v>
+      </x:c>
+      <x:c r="O92" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P92" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q92" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R92" s="3" t="str">
+        <x:v>39c6e94b90f61a66ffdeda4605a7ec972053bfa3f4110036575f7ef54c4c2ad5</x:v>
+      </x:c>
+      <x:c r="S92" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="40" customHeight="1">
+      <x:c r="A93" s="3" t="str">
+        <x:v>LIC2026-IMG2547</x:v>
+      </x:c>
+      <x:c r="B93" s="3" t="str">
+        <x:v>Mi è piaciuta tantissimo</x:v>
+      </x:c>
+      <x:c r="C93" s="3" t="str">
+        <x:v>Molto interessante</x:v>
+      </x:c>
+      <x:c r="D93" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="E93" s="3" t="str">
+        <x:v>Più curioso/a</x:v>
+      </x:c>
+      <x:c r="F93" s="3" t="str">
+        <x:v>Più interessato/a</x:v>
+      </x:c>
+      <x:c r="G93" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="H93" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I93" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J93" s="3" t="str">
+        <x:v>Femminile</x:v>
+      </x:c>
+      <x:c r="K93" s="3" t="str">
+        <x:v>26–40</x:v>
+      </x:c>
+      <x:c r="L93" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="M93" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 103</x:v>
+      </x:c>
+      <x:c r="N93" s="3" t="str">
+        <x:v>IMG_2547.JPG</x:v>
+      </x:c>
+      <x:c r="O93" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P93" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q93" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R93" s="3" t="str">
+        <x:v>8e4bc77eaa157abf78362346ab5b685b29178d1a5d787888353f6d013a4b43f3</x:v>
+      </x:c>
+      <x:c r="S93" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="40" customHeight="1">
+      <x:c r="A94" s="3" t="str">
+        <x:v>LIC2026-IMG2548</x:v>
+      </x:c>
+      <x:c r="B94" s="3" t="str">
+        <x:v>Mi è piaciuta</x:v>
+      </x:c>
+      <x:c r="C94" s="3" t="str">
+        <x:v>COINVOLGENTE, DIVERTENTE,</x:v>
+      </x:c>
+      <x:c r="D94" s="3" t="str">
+        <x:v>Sì, un po’</x:v>
+      </x:c>
+      <x:c r="E94" s="3" t="str">
+        <x:v>Più curioso/a</x:v>
+      </x:c>
+      <x:c r="F94" s="3" t="str">
+        <x:v>Più interessato/a</x:v>
+      </x:c>
+      <x:c r="G94" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="H94" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I94" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J94" s="3" t="str">
+        <x:v>Maschile</x:v>
+      </x:c>
+      <x:c r="K94" s="3" t="str">
+        <x:v>11–14</x:v>
+      </x:c>
+      <x:c r="L94" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="M94" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 102</x:v>
+      </x:c>
+      <x:c r="N94" s="3" t="str">
+        <x:v>IMG_2548.JPG</x:v>
+      </x:c>
+      <x:c r="O94" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P94" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q94" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R94" s="3" t="str">
+        <x:v>c2c312252916c60bf1df2a68edd1ff2f54559f9374e52a2fda95885f4643fa13</x:v>
+      </x:c>
+      <x:c r="S94" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="40" customHeight="1">
+      <x:c r="A95" s="3" t="str">
+        <x:v>LIC2026-IMG2549</x:v>
+      </x:c>
+      <x:c r="B95" s="3" t="str">
+        <x:v>Mi è piaciuta</x:v>
+      </x:c>
+      <x:c r="C95" s="3" t="str">
+        <x:v>BELLO, INTERESSANTE</x:v>
+      </x:c>
+      <x:c r="D95" s="3" t="str">
+        <x:v>Sì, un po’</x:v>
+      </x:c>
+      <x:c r="E95" s="3" t="str">
+        <x:v>Più curioso/a</x:v>
+      </x:c>
+      <x:c r="F95" s="3" t="str">
+        <x:v>Più interessato/a</x:v>
+      </x:c>
+      <x:c r="G95" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="H95" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I95" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J95" s="3" t="str">
+        <x:v>Maschile</x:v>
+      </x:c>
+      <x:c r="K95" s="3" t="str">
+        <x:v>11–14</x:v>
+      </x:c>
+      <x:c r="L95" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="M95" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 101</x:v>
+      </x:c>
+      <x:c r="N95" s="3" t="str">
+        <x:v>IMG_2549.JPG</x:v>
+      </x:c>
+      <x:c r="O95" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P95" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q95" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R95" s="3" t="str">
+        <x:v>47091d3b0b5b7461094d8a2503f62279b93a5b94baac4ad31154b9fc41a41881</x:v>
+      </x:c>
+      <x:c r="S95" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="40" customHeight="1">
+      <x:c r="A96" s="3" t="str">
+        <x:v>LIC2026-IMG2550</x:v>
+      </x:c>
+      <x:c r="B96" s="3" t="str">
+        <x:v>Mi è piaciuta tantissimo</x:v>
+      </x:c>
+      <x:c r="C96" s="3" t="str"/>
+      <x:c r="D96" s="3" t="str">
+        <x:v>Sì, un po’</x:v>
+      </x:c>
+      <x:c r="E96" s="3" t="str">
+        <x:v>Più curioso/a</x:v>
+      </x:c>
+      <x:c r="F96" s="3" t="str">
+        <x:v>Più interessato/a</x:v>
+      </x:c>
+      <x:c r="G96" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="H96" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I96" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J96" s="3" t="str">
+        <x:v>Maschile</x:v>
+      </x:c>
+      <x:c r="K96" s="3" t="str">
+        <x:v>41–60</x:v>
+      </x:c>
+      <x:c r="L96" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="M96" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 100
+Q2: Risposta non compilata nella fotografia.</x:v>
+      </x:c>
+      <x:c r="N96" s="3" t="str">
+        <x:v>IMG_2550.JPG</x:v>
+      </x:c>
+      <x:c r="O96" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P96" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q96" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R96" s="3" t="str">
+        <x:v>5a80b6ca87f516168f43ca2436772b5d04c5baf842ba381b44e85ff35cf54253</x:v>
+      </x:c>
+      <x:c r="S96" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="40" customHeight="1">
+      <x:c r="A97" s="3" t="str">
+        <x:v>LIC2026-IMG2553</x:v>
+      </x:c>
+      <x:c r="B97" s="3" t="str">
+        <x:v>Mi è piaciuta tantissimo</x:v>
+      </x:c>
+      <x:c r="C97" s="3" t="str">
+        <x:v>bella, interessante, coinvolgente</x:v>
+      </x:c>
+      <x:c r="D97" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="E97" s="3" t="str">
+        <x:v>Più curioso/a</x:v>
+      </x:c>
+      <x:c r="F97" s="3" t="str">
+        <x:v>Più interessato/a</x:v>
+      </x:c>
+      <x:c r="G97" s="3" t="str">
+        <x:v>In parte</x:v>
+      </x:c>
+      <x:c r="H97" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I97" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J97" s="3" t="str">
+        <x:v>Maschile</x:v>
+      </x:c>
+      <x:c r="K97" s="3" t="str">
+        <x:v>Meno di 11</x:v>
+      </x:c>
+      <x:c r="L97" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="M97" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 99</x:v>
+      </x:c>
+      <x:c r="N97" s="3" t="str">
+        <x:v>IMG_2553.JPG</x:v>
+      </x:c>
+      <x:c r="O97" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P97" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q97" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R97" s="3" t="str">
+        <x:v>0885cbfa28cfadc7a33ceb46d89c9ae012dd1a18ce848fecbb70fef5b46ca4fa</x:v>
+      </x:c>
+      <x:c r="S97" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="40" customHeight="1">
+      <x:c r="A98" s="3" t="str">
+        <x:v>LIC2026-IMG2554</x:v>
+      </x:c>
+      <x:c r="B98" s="3" t="str">
+        <x:v>Mi è piaciuta tantissimo</x:v>
+      </x:c>
+      <x:c r="C98" s="3" t="str">
+        <x:v>RAGIONAMENTO, ATTENZIONE, SCOPERTA</x:v>
+      </x:c>
+      <x:c r="D98" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="E98" s="3" t="str">
+        <x:v>Più curioso/a</x:v>
+      </x:c>
+      <x:c r="F98" s="3" t="str">
+        <x:v>Interessato/a come prima</x:v>
+      </x:c>
+      <x:c r="G98" s="3" t="str">
+        <x:v>In parte</x:v>
+      </x:c>
+      <x:c r="H98" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I98" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J98" s="3" t="str">
+        <x:v>Maschile</x:v>
+      </x:c>
+      <x:c r="K98" s="3" t="str">
+        <x:v>11–14</x:v>
+      </x:c>
+      <x:c r="L98" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="M98" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 98</x:v>
+      </x:c>
+      <x:c r="N98" s="3" t="str">
+        <x:v>IMG_2554.JPG</x:v>
+      </x:c>
+      <x:c r="O98" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P98" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q98" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R98" s="3" t="str">
+        <x:v>d0adecf6d4e98249d0896f70a0484e7442dabf233ecc7a565cc5ca52d9283339</x:v>
+      </x:c>
+      <x:c r="S98" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="40" customHeight="1">
+      <x:c r="A99" s="3" t="str">
+        <x:v>LIC2026-IMG2555</x:v>
+      </x:c>
+      <x:c r="B99" s="3" t="str">
+        <x:v>Mi è piaciuta</x:v>
+      </x:c>
+      <x:c r="C99" s="3" t="str">
+        <x:v>DIVULGATIVA</x:v>
+      </x:c>
+      <x:c r="D99" s="3" t="str">
+        <x:v>Sì, un po’</x:v>
+      </x:c>
+      <x:c r="E99" s="3" t="str">
+        <x:v>Più curioso/a</x:v>
+      </x:c>
+      <x:c r="F99" s="3" t="str">
+        <x:v>Più interessato/a</x:v>
+      </x:c>
+      <x:c r="G99" s="3" t="str">
+        <x:v>In parte</x:v>
+      </x:c>
+      <x:c r="H99" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I99" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J99" s="3" t="str">
+        <x:v>Femminile</x:v>
+      </x:c>
+      <x:c r="K99" s="3" t="str">
+        <x:v>26–40</x:v>
+      </x:c>
+      <x:c r="L99" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="M99" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 97</x:v>
+      </x:c>
+      <x:c r="N99" s="3" t="str">
+        <x:v>IMG_2555.JPG</x:v>
+      </x:c>
+      <x:c r="O99" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P99" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q99" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R99" s="3" t="str">
+        <x:v>f23a95c43b636f6e5d334d913403d3853db807b3bac38ca002e770e08be501d5</x:v>
+      </x:c>
+      <x:c r="S99" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="40" customHeight="1">
+      <x:c r="A100" s="3" t="str">
+        <x:v>LIC2026-IMG2556</x:v>
+      </x:c>
+      <x:c r="B100" s="3" t="str">
+        <x:v>Mi è piaciuta</x:v>
+      </x:c>
+      <x:c r="C100" s="3" t="str">
+        <x:v>INTERATTIVA</x:v>
+      </x:c>
+      <x:c r="D100" s="3" t="str">
+        <x:v>Sì, un po’</x:v>
+      </x:c>
+      <x:c r="E100" s="3" t="str">
+        <x:v>Curioso/a come prima</x:v>
+      </x:c>
+      <x:c r="F100" s="3" t="str">
+        <x:v>Interessato/a come prima</x:v>
+      </x:c>
+      <x:c r="G100" s="3" t="str">
+        <x:v>In parte</x:v>
+      </x:c>
+      <x:c r="H100" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I100" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J100" s="3" t="str">
+        <x:v>Femminile</x:v>
+      </x:c>
+      <x:c r="K100" s="3" t="str">
+        <x:v>19–25</x:v>
+      </x:c>
+      <x:c r="L100" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="M100" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 96</x:v>
+      </x:c>
+      <x:c r="N100" s="3" t="str">
+        <x:v>IMG_2556.JPG</x:v>
+      </x:c>
+      <x:c r="O100" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P100" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q100" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R100" s="3" t="str">
+        <x:v>03c2cdf1e99a2adad78fa8de9cc0dc926322f997aebc490d758e8899fd386776</x:v>
+      </x:c>
+      <x:c r="S100" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="40" customHeight="1">
+      <x:c r="A101" s="3" t="str">
+        <x:v>LIC2026-IMG2557</x:v>
+      </x:c>
+      <x:c r="B101" s="3" t="str">
+        <x:v>Mi è piaciuta</x:v>
+      </x:c>
+      <x:c r="C101" s="3" t="str">
+        <x:v>ORIGINALE, COINVOLGENTE</x:v>
+      </x:c>
+      <x:c r="D101" s="3" t="str">
+        <x:v>Sì, un po’</x:v>
+      </x:c>
+      <x:c r="E101" s="3" t="str">
+        <x:v>Più curioso/a</x:v>
+      </x:c>
+      <x:c r="F101" s="3" t="str">
+        <x:v>Più interessato/a</x:v>
+      </x:c>
+      <x:c r="G101" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="H101" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I101" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J101" s="3" t="str">
+        <x:v>Femminile</x:v>
+      </x:c>
+      <x:c r="K101" s="3" t="str">
+        <x:v>15–18</x:v>
+      </x:c>
+      <x:c r="L101" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="M101" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 95</x:v>
+      </x:c>
+      <x:c r="N101" s="3" t="str">
+        <x:v>IMG_2557.JPG</x:v>
+      </x:c>
+      <x:c r="O101" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P101" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q101" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R101" s="3" t="str">
+        <x:v>26825845f8c55c08c415b09d2b155b65bee398d57c48d9611ef82bb02f283921</x:v>
+      </x:c>
+      <x:c r="S101" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="40" customHeight="1">
+      <x:c r="A102" s="3" t="str">
+        <x:v>LIC2026-IMG2558</x:v>
+      </x:c>
+      <x:c r="B102" s="3" t="str">
+        <x:v>Mi è piaciuta</x:v>
+      </x:c>
+      <x:c r="C102" s="3" t="str">
+        <x:v>Interessante</x:v>
+      </x:c>
+      <x:c r="D102" s="3" t="str">
+        <x:v>Sì, un po’</x:v>
+      </x:c>
+      <x:c r="E102" s="3" t="str">
+        <x:v>Curioso/a come prima</x:v>
+      </x:c>
+      <x:c r="F102" s="3" t="str">
+        <x:v>Interessato/a come prima</x:v>
+      </x:c>
+      <x:c r="G102" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="H102" s="3" t="str">
+        <x:v>A volte</x:v>
+      </x:c>
+      <x:c r="I102" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J102" s="3" t="str">
+        <x:v>Maschile</x:v>
+      </x:c>
+      <x:c r="K102" s="3" t="str">
+        <x:v>19–25</x:v>
+      </x:c>
+      <x:c r="L102" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="M102" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 94</x:v>
+      </x:c>
+      <x:c r="N102" s="3" t="str">
+        <x:v>IMG_2558.JPG</x:v>
+      </x:c>
+      <x:c r="O102" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P102" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q102" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R102" s="3" t="str">
+        <x:v>e94299be53821ea5d29fa4f82ed428176c4e10d4b196e0fd9a2b60153e03e685</x:v>
+      </x:c>
+      <x:c r="S102" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="40" customHeight="1">
+      <x:c r="A103" s="3" t="str">
+        <x:v>LIC2026-IMG2559</x:v>
+      </x:c>
+      <x:c r="B103" s="3" t="str">
+        <x:v>Mi è piaciuta</x:v>
+      </x:c>
+      <x:c r="C103" s="3" t="str"/>
+      <x:c r="D103" s="3" t="str">
+        <x:v>Sì, un po’</x:v>
+      </x:c>
+      <x:c r="E103" s="3" t="str">
+        <x:v>Curioso/a come prima</x:v>
+      </x:c>
+      <x:c r="F103" s="3" t="str">
+        <x:v>Interessato/a come prima</x:v>
+      </x:c>
+      <x:c r="G103" s="3" t="str">
+        <x:v>In parte</x:v>
+      </x:c>
+      <x:c r="H103" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I103" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J103" s="3" t="str">
+        <x:v>Femminile</x:v>
+      </x:c>
+      <x:c r="K103" s="3" t="str">
+        <x:v>41–60</x:v>
+      </x:c>
+      <x:c r="L103" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="M103" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 93
+Q2: Risposta non compilata nella fotografia.</x:v>
+      </x:c>
+      <x:c r="N103" s="3" t="str">
+        <x:v>IMG_2559.JPG</x:v>
+      </x:c>
+      <x:c r="O103" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P103" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q103" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R103" s="3" t="str">
+        <x:v>31d1e37d332654f351e6a7ee5b8baea08df62029fa70b4e839e09a9ac5cbd4a1</x:v>
+      </x:c>
+      <x:c r="S103" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="40" customHeight="1">
+      <x:c r="A104" s="3" t="str">
+        <x:v>LIC2026-IMG2560</x:v>
+      </x:c>
+      <x:c r="B104" s="3" t="str">
+        <x:v>Mi è piaciuta tantissimo</x:v>
+      </x:c>
+      <x:c r="C104" s="3" t="str">
+        <x:v>divertente, educativa</x:v>
+      </x:c>
+      <x:c r="D104" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="E104" s="3" t="str">
+        <x:v>Curioso/a come prima</x:v>
+      </x:c>
+      <x:c r="F104" s="3" t="str">
+        <x:v>Interessato/a come prima</x:v>
+      </x:c>
+      <x:c r="G104" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="H104" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I104" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J104" s="3" t="str">
+        <x:v>Altro</x:v>
+      </x:c>
+      <x:c r="K104" s="3" t="str">
+        <x:v>15–18</x:v>
+      </x:c>
+      <x:c r="L104" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="M104" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 92</x:v>
+      </x:c>
+      <x:c r="N104" s="3" t="str">
+        <x:v>IMG_2560.JPG</x:v>
+      </x:c>
+      <x:c r="O104" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P104" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q104" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R104" s="3" t="str">
+        <x:v>9e58d1775e71d320082137d88175930906640d302bc8d57e3ba84e45b8ae2121</x:v>
+      </x:c>
+      <x:c r="S104" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="40" customHeight="1">
+      <x:c r="A105" s="3" t="str">
+        <x:v>LIC2026-IMG2561</x:v>
+      </x:c>
+      <x:c r="B105" s="3" t="str">
+        <x:v>Mi è piaciuta tantissimo</x:v>
+      </x:c>
+      <x:c r="C105" s="3" t="str">
+        <x:v>DIVERTENTE, STIMOLANTE</x:v>
+      </x:c>
+      <x:c r="D105" s="3" t="str">
+        <x:v>Sì, un po’</x:v>
+      </x:c>
+      <x:c r="E105" s="3" t="str">
+        <x:v>Più curioso/a</x:v>
+      </x:c>
+      <x:c r="F105" s="3" t="str">
+        <x:v>Più interessato/a</x:v>
+      </x:c>
+      <x:c r="G105" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="H105" s="3" t="str">
+        <x:v>A volte</x:v>
+      </x:c>
+      <x:c r="I105" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J105" s="3" t="str">
+        <x:v>Femminile</x:v>
+      </x:c>
+      <x:c r="K105" s="3" t="str">
+        <x:v>41–60</x:v>
+      </x:c>
+      <x:c r="L105" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="M105" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 91</x:v>
+      </x:c>
+      <x:c r="N105" s="3" t="str">
+        <x:v>IMG_2561.JPG</x:v>
+      </x:c>
+      <x:c r="O105" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P105" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q105" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R105" s="3" t="str">
+        <x:v>65007904d7d4036da4319672f7cc5a6185b0b4a7b4156f2c1e0db75d606e7462</x:v>
+      </x:c>
+      <x:c r="S105" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="40" customHeight="1">
+      <x:c r="A106" s="3" t="str">
+        <x:v>LIC2026-IMG2562</x:v>
+      </x:c>
+      <x:c r="B106" s="3" t="str">
+        <x:v>Non mi è piaciuta molto</x:v>
+      </x:c>
+      <x:c r="C106" s="3" t="str"/>
+      <x:c r="D106" s="3" t="str">
+        <x:v>Sì, un po’</x:v>
+      </x:c>
+      <x:c r="E106" s="3" t="str">
+        <x:v>Curioso/a come prima</x:v>
+      </x:c>
+      <x:c r="F106" s="3" t="str">
+        <x:v>Interessato/a come prima</x:v>
+      </x:c>
+      <x:c r="G106" s="3" t="str">
+        <x:v>In parte</x:v>
+      </x:c>
+      <x:c r="H106" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I106" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J106" s="3" t="str">
+        <x:v>Femminile</x:v>
+      </x:c>
+      <x:c r="K106" s="3" t="str">
+        <x:v>15–18</x:v>
+      </x:c>
+      <x:c r="L106" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="M106" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 90
+Q2: Risposta non compilata nella fotografia.</x:v>
+      </x:c>
+      <x:c r="N106" s="3" t="str">
+        <x:v>IMG_2562.JPG</x:v>
+      </x:c>
+      <x:c r="O106" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P106" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q106" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R106" s="3" t="str">
+        <x:v>fd241a04c18dd4684b0ebbf3bed83814745dedd8b3d6ed56d8340881c8b37253</x:v>
+      </x:c>
+      <x:c r="S106" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="40" customHeight="1">
+      <x:c r="A107" s="3" t="str">
+        <x:v>LIC2026-IMG2563</x:v>
+      </x:c>
+      <x:c r="B107" s="3" t="str">
+        <x:v>Mi è piaciuta</x:v>
+      </x:c>
+      <x:c r="C107" s="3" t="str"/>
+      <x:c r="D107" s="3" t="str">
+        <x:v>Sì, un po’</x:v>
+      </x:c>
+      <x:c r="E107" s="3" t="str">
+        <x:v>Curioso/a come prima</x:v>
+      </x:c>
+      <x:c r="F107" s="3" t="str">
+        <x:v>Interessato/a come prima</x:v>
+      </x:c>
+      <x:c r="G107" s="3" t="str">
+        <x:v>In parte</x:v>
+      </x:c>
+      <x:c r="H107" s="3" t="str">
+        <x:v>A volte</x:v>
+      </x:c>
+      <x:c r="I107" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J107" s="3" t="str">
+        <x:v>Altro</x:v>
+      </x:c>
+      <x:c r="K107" s="3" t="str">
+        <x:v>15–18</x:v>
+      </x:c>
+      <x:c r="L107" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="M107" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 89
+Q2: Risposta non compilata nella fotografia.</x:v>
+      </x:c>
+      <x:c r="N107" s="3" t="str">
+        <x:v>IMG_2563.JPG</x:v>
+      </x:c>
+      <x:c r="O107" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P107" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q107" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R107" s="3" t="str">
+        <x:v>8f46d4b5bc95b6a0fce441dd5e8f7cad9a7f80cfe7ded8710a56402e43385bcc</x:v>
+      </x:c>
+      <x:c r="S107" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="40" customHeight="1">
+      <x:c r="A108" s="3" t="str">
+        <x:v>LIC2026-IMG2564</x:v>
+      </x:c>
+      <x:c r="B108" s="3" t="str">
+        <x:v>Mi è piaciuta</x:v>
+      </x:c>
+      <x:c r="C108" s="3" t="str">
+        <x:v>DIVERTENTE, COLLABORATIVA</x:v>
+      </x:c>
+      <x:c r="D108" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="E108" s="3" t="str">
+        <x:v>Curioso/a come prima</x:v>
+      </x:c>
+      <x:c r="F108" s="3" t="str">
+        <x:v>Interessato/a come prima</x:v>
+      </x:c>
+      <x:c r="G108" s="3" t="str">
+        <x:v>In parte</x:v>
+      </x:c>
+      <x:c r="H108" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I108" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J108" s="3" t="str">
+        <x:v>Maschile</x:v>
+      </x:c>
+      <x:c r="K108" s="3" t="str">
+        <x:v>19–25</x:v>
+      </x:c>
+      <x:c r="L108" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="M108" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 88</x:v>
+      </x:c>
+      <x:c r="N108" s="3" t="str">
+        <x:v>IMG_2564.JPG</x:v>
+      </x:c>
+      <x:c r="O108" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P108" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q108" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R108" s="3" t="str">
+        <x:v>03d9bd4ade77e328a4a5b973a99287274c07b7e92a8f3da9a4359373f5ffdac1</x:v>
+      </x:c>
+      <x:c r="S108" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="40" customHeight="1">
+      <x:c r="A109" s="3" t="str">
+        <x:v>LIC2026-IMG2565</x:v>
+      </x:c>
+      <x:c r="B109" s="3" t="str">
+        <x:v>Mi è piaciuta tantissimo</x:v>
+      </x:c>
+      <x:c r="C109" s="3" t="str"/>
+      <x:c r="D109" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="E109" s="3" t="str">
+        <x:v>Più curioso/a</x:v>
+      </x:c>
+      <x:c r="F109" s="3" t="str">
+        <x:v>Più interessato/a</x:v>
+      </x:c>
+      <x:c r="G109" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="H109" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I109" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J109" s="3" t="str">
+        <x:v>Femminile</x:v>
+      </x:c>
+      <x:c r="K109" s="3" t="str">
+        <x:v>26–40</x:v>
+      </x:c>
+      <x:c r="L109" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="M109" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 87
+Q2: Risposta non compilata nella fotografia.</x:v>
+      </x:c>
+      <x:c r="N109" s="3" t="str">
+        <x:v>IMG_2565.JPG</x:v>
+      </x:c>
+      <x:c r="O109" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P109" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q109" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R109" s="3" t="str">
+        <x:v>4b782e4dfb539c17c60f3bd8b6830e6e51ae3d0fbe7ac4b325533e562ef3c71c</x:v>
+      </x:c>
+      <x:c r="S109" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="52" customHeight="1">
+      <x:c r="A110" s="3" t="str">
+        <x:v>LIC2026-IMG2566</x:v>
+      </x:c>
+      <x:c r="B110" s="3" t="str">
+        <x:v>Mi è piaciuta tantissimo</x:v>
+      </x:c>
+      <x:c r="C110" s="3" t="str">
+        <x:v>DIVERTENTE EDUCATIVA</x:v>
+      </x:c>
+      <x:c r="D110" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="E110" s="3" t="str">
+        <x:v>Curioso/a come prima</x:v>
+      </x:c>
+      <x:c r="F110" s="3" t="str">
+        <x:v>Più interessato/a</x:v>
+      </x:c>
+      <x:c r="G110" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="H110" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I110" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J110" s="3" t="str">
+        <x:v>Femminile</x:v>
+      </x:c>
+      <x:c r="K110" s="3" t="str">
+        <x:v>11–14</x:v>
+      </x:c>
+      <x:c r="L110" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="M110" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 86
+duplicato: IMG_2567.JPG fotografa la stessa scheda: conteggiata una sola volta.</x:v>
+      </x:c>
+      <x:c r="N110" s="3" t="str">
+        <x:v>IMG_2566.JPG</x:v>
+      </x:c>
+      <x:c r="O110" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P110" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q110" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R110" s="3" t="str">
+        <x:v>213b51a94549ce53316edc360a4ceb3423a8f4ee1a698e046a97f89df3283922</x:v>
+      </x:c>
+      <x:c r="S110" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="52" customHeight="1">
+      <x:c r="A111" s="3" t="str">
+        <x:v>LIC2026-IMG2568</x:v>
+      </x:c>
+      <x:c r="B111" s="3" t="str">
+        <x:v>Mi è piaciuta tantissimo</x:v>
+      </x:c>
+      <x:c r="C111" s="3" t="str">
+        <x:v>FIGO ASSAI</x:v>
+      </x:c>
+      <x:c r="D111" s="3" t="str">
+        <x:v>Sì, un po’</x:v>
+      </x:c>
+      <x:c r="E111" s="3" t="str">
+        <x:v>Curioso/a come prima</x:v>
+      </x:c>
+      <x:c r="F111" s="3" t="str">
+        <x:v>Interessato/a come prima</x:v>
+      </x:c>
+      <x:c r="G111" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="H111" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I111" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J111" s="3" t="str">
+        <x:v>Maschile</x:v>
+      </x:c>
+      <x:c r="K111" s="3" t="str">
+        <x:v>19–25</x:v>
+      </x:c>
+      <x:c r="L111" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="M111" s="3" t="str">
+        <x:v>scheda: Numero manoscritto leggibile come 80; conservato senza rinumerare. Foto distinta dalle precedenti.</x:v>
+      </x:c>
+      <x:c r="N111" s="3" t="str">
+        <x:v>IMG_2568.JPG</x:v>
+      </x:c>
+      <x:c r="O111" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P111" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q111" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R111" s="3" t="str">
+        <x:v>7d145725bc8663f5fe29910c3a992d8e68c937767411dcd76a01e01c8e01407c</x:v>
+      </x:c>
+      <x:c r="S111" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="40" customHeight="1">
+      <x:c r="A112" s="3" t="str">
+        <x:v>LIC2026-IMG2570</x:v>
+      </x:c>
+      <x:c r="B112" s="3" t="str">
+        <x:v>Mi è piaciuta tantissimo</x:v>
+      </x:c>
+      <x:c r="C112" s="3" t="str">
+        <x:v>INGEGNERISTICA SUPER QUARK</x:v>
+      </x:c>
+      <x:c r="D112" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="E112" s="3" t="str">
+        <x:v>Più curioso/a</x:v>
+      </x:c>
+      <x:c r="F112" s="3" t="str">
+        <x:v>Più interessato/a</x:v>
+      </x:c>
+      <x:c r="G112" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="H112" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I112" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="J112" s="3" t="str">
+        <x:v>Maschile</x:v>
+      </x:c>
+      <x:c r="K112" s="3" t="str">
+        <x:v>19–25</x:v>
+      </x:c>
+      <x:c r="L112" s="3" t="str">
+        <x:v>Sì</x:v>
+      </x:c>
+      <x:c r="M112" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 84</x:v>
+      </x:c>
+      <x:c r="N112" s="3" t="str">
+        <x:v>IMG_2570.JPG</x:v>
+      </x:c>
+      <x:c r="O112" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P112" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q112" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R112" s="3" t="str">
+        <x:v>bbdf67ee3dffb859c8ed0aebbdb931dec461b2324bbfeb5a29fafaabb4dd78ed</x:v>
+      </x:c>
+      <x:c r="S112" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="40" customHeight="1">
+      <x:c r="A113" s="3" t="str">
+        <x:v>LIC2026-IMG2571</x:v>
+      </x:c>
+      <x:c r="B113" s="3" t="str">
+        <x:v>Mi è piaciuta</x:v>
+      </x:c>
+      <x:c r="C113" s="3" t="str">
+        <x:v>BELLA CURIOSA DIVERTENTE</x:v>
+      </x:c>
+      <x:c r="D113" s="3" t="str">
+        <x:v>Sì, un po’</x:v>
+      </x:c>
+      <x:c r="E113" s="3" t="str">
+        <x:v>Più curioso/a</x:v>
+      </x:c>
+      <x:c r="F113" s="3" t="str">
+        <x:v>Interessato/a come prima</x:v>
+      </x:c>
+      <x:c r="G113" s="3" t="str">
+        <x:v>In parte</x:v>
+      </x:c>
+      <x:c r="H113" s="3" t="str">
+        <x:v>A volte</x:v>
+      </x:c>
+      <x:c r="I113" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J113" s="3" t="str">
+        <x:v>Femminile</x:v>
+      </x:c>
+      <x:c r="K113" s="3" t="str">
+        <x:v>11–14</x:v>
+      </x:c>
+      <x:c r="L113" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="M113" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 83</x:v>
+      </x:c>
+      <x:c r="N113" s="3" t="str">
+        <x:v>IMG_2571.JPG</x:v>
+      </x:c>
+      <x:c r="O113" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P113" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q113" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R113" s="3" t="str">
+        <x:v>cfe25e5742bac4e4f51ea4643c76d0d514ce1238a1499ca85cc1ae2e3b7c0e0e</x:v>
+      </x:c>
+      <x:c r="S113" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="52" customHeight="1">
+      <x:c r="A114" s="3" t="str">
+        <x:v>LIC2026-IMG2572</x:v>
+      </x:c>
+      <x:c r="B114" s="3" t="str">
+        <x:v>Mi è piaciuta tantissimo</x:v>
+      </x:c>
+      <x:c r="C114" s="3" t="str"/>
+      <x:c r="D114" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="E114" s="3" t="str">
+        <x:v>Più curioso/a</x:v>
+      </x:c>
+      <x:c r="F114" s="3" t="str">
+        <x:v>Più interessato/a</x:v>
+      </x:c>
+      <x:c r="G114" s="3" t="str">
+        <x:v>Sì, molto</x:v>
+      </x:c>
+      <x:c r="H114" s="3" t="str">
+        <x:v>Mai</x:v>
+      </x:c>
+      <x:c r="I114" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J114" s="3" t="str">
+        <x:v>Femminile</x:v>
+      </x:c>
+      <x:c r="K114" s="3" t="str">
+        <x:v>41–60</x:v>
+      </x:c>
+      <x:c r="L114" s="3" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="M114" s="3" t="str">
+        <x:v>scheda: Numero manoscritto: 82; scheda distinta dalla precedente 82 (IMG_2423.JPG).
+Q2: Risposta non compilata nella fotografia.</x:v>
+      </x:c>
+      <x:c r="N114" s="3" t="str">
+        <x:v>IMG_2572.JPG</x:v>
+      </x:c>
+      <x:c r="O114" s="3" t="str">
+        <x:v>Potenza</x:v>
+      </x:c>
+      <x:c r="P114" s="3" t="str">
+        <x:v>Roma</x:v>
+      </x:c>
+      <x:c r="Q114" s="3" t="str">
+        <x:v>Confermata</x:v>
+      </x:c>
+      <x:c r="R114" s="3" t="str">
+        <x:v>33718fede21ff82b7fabb78f7cfdec0bc25126799694c199d54cbd07d77b1120</x:v>
+      </x:c>
+      <x:c r="S114" s="3" t="str">
+        <x:v>Lucania is comics</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc584ac3919a84e1e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f1c561b89c0482a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>